<commit_message>
Rasid demo: anonymise sample report (report.xlsx)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demos/rasid-checker/report.xlsx
+++ b/demos/rasid-checker/report.xlsx
@@ -552,7 +552,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.visiondentalclinic.com/</t>
+          <t>https://site-01.example/</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -565,12 +565,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://visiondentalclinic.com/</t>
+          <t>https://site-01.example/</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.visiondentalclinic.com/ → https://visiondentalclinic.com/</t>
+          <t>https://site-01.example/ → https://site-01.example/</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -586,7 +586,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Dental Clinic in Abu Dhabi – Vision Dental Clinic</t>
+          <t>موقع تجريبي 01</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://meddental.ae/</t>
+          <t>https://site-02.example/</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -632,12 +632,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.meddental.ae/</t>
+          <t>https://site-02.example/</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://meddental.ae/ → https://www.meddental.ae/</t>
+          <t>https://site-02.example/ → https://site-02.example/</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -653,7 +653,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Dental Clinic in JLT Dubai | The Dome MedDental Clinic</t>
+          <t>موقع تجريبي 02</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://vistaoman.com/</t>
+          <t>https://site-03.example/</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://vistaoman.com/</t>
+          <t>https://site-03.example/</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -712,7 +712,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Vista Real Estate - Most Trusted Real Estate Company in Oman</t>
+          <t>موقع تجريبي 03</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -741,7 +741,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://zahrabeautysalon.qa/</t>
+          <t>https://site-04.example/</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://zahrabeautysalon.qa/</t>
+          <t>https://site-04.example/</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -771,7 +771,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Zahra Beauty Salon and Spa | Experience the Ultimate in Beauty and Relaxation in Doha, Qatar.</t>
+          <t>موقع تجريبي 04</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -800,7 +800,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.arizonahomesbh.com/</t>
+          <t>https://site-05.example/</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.arizonahomesbh.com/</t>
+          <t>https://site-05.example/</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -830,7 +830,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Best Real Estate Agent In Manama, Bahrain | Villa For Rent In Bahrain</t>
+          <t>موقع تجريبي 05</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -859,7 +859,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://houseofamal.net/</t>
+          <t>https://site-06.example/</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://houseofamal.net/</t>
+          <t>https://site-06.example/</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
@@ -889,7 +889,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Too many requests</t>
+          <t>موقع تجريبي 06</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -916,7 +916,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.semiramiscatering.com/</t>
+          <t>https://site-07.example/</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.semiramiscatering.com/</t>
+          <t>https://site-07.example/</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -946,7 +946,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Home - Simramis Catering</t>
+          <t>موقع تجريبي 07</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -979,7 +979,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://royalcaters.co/</t>
+          <t>https://site-08.example/</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -992,7 +992,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://royalcaters.co/</t>
+          <t>https://site-08.example/</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Royal Caters - Kuwait</t>
+          <t>موقع تجريبي 08</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://grandpachef.ae/</t>
+          <t>https://site-09.example/</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://grandpachef.ae/</t>
+          <t>https://site-09.example/</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Best Restaurant in Sharjah | Grandpa Chef</t>
+          <t>موقع تجريبي 09</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1099,14 +1099,14 @@
       <c r="O10" s="3" t="inlineStr">
         <is>
           <t>slow response (6.2s)
-broken WhatsApp link: https://wa.me/+971%2056%20300%205790 (number contains spaces/dashes, WhatsApp needs digits only (+971 56 300 5790))</t>
+broken WhatsApp link: https://wa.me/+971%2056%20300%200000 (number contains spaces/dashes, WhatsApp needs digits only (+971 56 300 0000))</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://sumo.sa/</t>
+          <t>https://site-10.example/</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://sumo.sa/</t>
+          <t>https://site-10.example/</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>عيادات السمو للعلاج الطبيعى</t>
+          <t>موقع تجريبي 10</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1165,7 +1165,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://riyadhluxurylive.com/</t>
+          <t>https://site-11.example/</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1178,12 +1178,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://riyadhluxurylive.com/ar/</t>
+          <t>https://site-11.example/ar/</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://riyadhluxurylive.com/ → https://riyadhluxurylive.com/ar/</t>
+          <t>https://site-11.example/ → https://site-11.example/ar/</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Riyadh Luxury</t>
+          <t>موقع تجريبي 11</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1228,7 +1228,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://heyaspa.com/</t>
+          <t>https://site-12.example/</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://heyaspa.com/</t>
+          <t>https://site-12.example/</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>الخدمات الرئيسيه فى هى سبا - heyaspa.com معهد صحى للسيدات</t>
+          <t>موقع تجريبي 12</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1287,7 +1287,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.wellmedbh.com/</t>
+          <t>https://site-13.example/</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.wellmedbh.com/</t>
+          <t>https://site-13.example/</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Wellmed Multi Specialty Center: Best Multispeciality Clinic Bahrain</t>
+          <t>موقع تجريبي 13</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1343,14 +1343,14 @@
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>broken internal link: https://www.wellmedbh.com/?page_id=14 (HTTP 404)</t>
+          <t>broken internal link: https://site-13.example/?page_id=14 (HTTP 404)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.iriswll.com/</t>
+          <t>https://site-14.example/</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.iriswll.com/</t>
+          <t>https://site-14.example/</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>IRIS Property Managers W.L.L | Property Management Company Bahrain</t>
+          <t>موقع تجريبي 14</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1409,7 +1409,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://loranclinics.com/</t>
+          <t>https://site-15.example/</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://loranclinics.com/</t>
+          <t>https://site-15.example/</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>افضل مستوصف اسنان في الرياض - اطلب الخدمه | Loran Clinics</t>
+          <t>موقع تجريبي 15</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1468,7 +1468,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://hairplayextensions.com/dubai/</t>
+          <t>https://site-16.example/dubai/</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://hairplayextensions.com/dubai/</t>
+          <t>https://site-16.example/dubai/</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Dubai Hair Extensions Salon | HAIRPLAY®</t>
+          <t>موقع تجريبي 16</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1527,7 +1527,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://blushncurls.ae/</t>
+          <t>https://site-17.example/</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://blushncurls.ae/</t>
+          <t>https://site-17.example/</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Best Ladies Salon &amp; Spa Near Me in Dubai - Beauty Salon in Al Barsha, Al Qusais &amp; Mankhool Dubai - Chemical Free Hair, Nails, Facials &amp; Bridal - Blush N Curls</t>
+          <t>موقع تجريبي 17</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1590,7 +1590,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://vog.ae/</t>
+          <t>https://site-18.example/</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://vog.ae/</t>
+          <t>https://site-18.example/</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Vog – Color your life</t>
+          <t>موقع تجريبي 18</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1654,7 +1654,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://crumbs.com.kw/</t>
+          <t>https://site-19.example/</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://crumbs.com.kw/</t>
+          <t>https://site-19.example/</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Crumbs</t>
+          <t>موقع تجريبي 19</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1713,7 +1713,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.25spaces.com/about-us</t>
+          <t>https://site-20.example/about-us</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.25spaces.com/about-us</t>
+          <t>https://site-20.example/about-us</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>About Us | 25 Spaces Real Estate | Luxury Properties in Doha, Qatar</t>
+          <t>موقع تجريبي 20</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1772,7 +1772,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://www.mycoreo.com/</t>
+          <t>https://site-21.example/</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.mycoreo.com/</t>
+          <t>https://site-21.example/</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -1802,7 +1802,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Property for Rent &amp; Sale in Qatar | Coreo Real Estate</t>
+          <t>موقع تجريبي 21</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1831,7 +1831,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://majestic.com.qa/</t>
+          <t>https://site-22.example/</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://majestic.com.qa/</t>
+          <t>https://site-22.example/</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Majestic Real Estate</t>
+          <t>موقع تجريبي 22</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1890,7 +1890,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://brightway.clinic/</t>
+          <t>https://site-23.example/</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://brightway.clinic/</t>
+          <t>https://site-23.example/</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Dental Services Clinic in Dubai | Digital Dentistry Near Me</t>
+          <t>موقع تجريبي 23</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1949,7 +1949,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://digitalimplantclinic.com/</t>
+          <t>https://site-24.example/</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://digitalimplantclinic.com/</t>
+          <t>https://site-24.example/</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
@@ -1979,7 +1979,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Dental Clinic in Dubai | Best Dentist in Dubai | Book Now</t>
+          <t>موقع تجريبي 24</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2008,7 +2008,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://dentaldate.ae/</t>
+          <t>https://site-25.example/</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://dentaldate.ae/</t>
+          <t>https://site-25.example/</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Best Dental Clinic in Dubai: Dentists in UAE</t>
+          <t>موقع تجريبي 25</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2067,7 +2067,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://professionalhaircenter.com/</t>
+          <t>https://site-26.example/</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://professionalhaircenter.com/</t>
+          <t>https://site-26.example/</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>مراكز بروفيشنال لتركيب الشعر في الإمارات | استبدال الشعر</t>
+          <t>موقع تجريبي 26</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2130,7 +2130,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.houseofbarber.com/</t>
+          <t>https://site-27.example/</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.houseofbarber.com/</t>
+          <t>https://site-27.example/</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>HOUSE OF BARBER - HOME</t>
+          <t>موقع تجريبي 27</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2189,7 +2189,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.bluechiphome.com/</t>
+          <t>https://site-28.example/</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.bluechiphome.com/</t>
+          <t>https://site-28.example/</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -2219,7 +2219,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Best Real Estate Agency in Dubai | Bluechip Real Estate</t>
+          <t>موقع تجريبي 28</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2246,14 +2246,14 @@
       <c r="O29" s="3" t="inlineStr">
         <is>
           <t>TLS certificate expires in 11 days
-broken WhatsApp link: https://wa.me/https://wa.link/4xi5xo (a URL pasted after wa.me/ instead of a number (https://wa.link/4xi5xo))</t>
+broken WhatsApp link: https://wa.me/https://site-29.example/4xi5xo (a URL pasted after wa.me/ instead of a number (https://site-29.example/4xi5xo))</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.yokosalonandspa.com/</t>
+          <t>https://site-30.example/</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.yokosalonandspa.com/</t>
+          <t>https://site-30.example/</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Coming Soon</t>
+          <t>موقع تجريبي 30</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2317,7 +2317,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.alanghamoman.com/</t>
+          <t>https://site-31.example/</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.alanghamoman.com/</t>
+          <t>https://site-31.example/</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Al Angham | Al Angham Restaurant</t>
+          <t>موقع تجريبي 31</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2380,7 +2380,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.noon.com/</t>
+          <t>https://site-32.example/</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.noon.com/</t>
+          <t>https://site-32.example/</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Access Denied</t>
+          <t>موقع تجريبي 32</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2437,7 +2437,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://www.namshi.com/</t>
+          <t>https://site-33.example/</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.namshi.com/</t>
+          <t>https://site-33.example/</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Access Denied</t>
+          <t>موقع تجريبي 33</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2494,7 +2494,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.jarir.com/</t>
+          <t>https://site-34.example/</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.jarir.com/</t>
+          <t>https://site-34.example/</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>مكتبة جرير، ليست مجرد مكتبة | السعودية</t>
+          <t>موقع تجريبي 34</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2553,7 +2553,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.extra.com/</t>
+          <t>https://site-35.example/</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -2566,12 +2566,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.extra.com/ar-sa</t>
+          <t>https://site-35.example/ar-sa</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.extra.com/ → https://www.extra.com/ar-sa/ → https://www.extra.com/ar-sa</t>
+          <t>https://site-35.example/ → https://site-35.example/ar-sa/ → https://site-35.example/ar-sa</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>إكسترا السعودية | اشترِ الإلكترونيات بثقة</t>
+          <t>موقع تجريبي 35</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2616,7 +2616,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.sharafdg.com/</t>
+          <t>https://site-36.example/</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.sharafdg.com/</t>
+          <t>https://site-36.example/</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Just a moment...</t>
+          <t>موقع تجريبي 36</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2673,7 +2673,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://www.xcite.com/</t>
+          <t>https://site-37.example/</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2686,12 +2686,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.xcite.com.sa/ar/sa-info</t>
+          <t>https://site-38.example/ar/sa-info</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.xcite.com/ → https://www.xcite.com.sa/ar → https://www.xcite.com.sa/ar/sa-info</t>
+          <t>https://site-37.example/ → https://site-38.example/ar → https://site-38.example/ar/sa-info</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2730,7 +2730,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.ounass.ae/</t>
+          <t>https://site-39.example/</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.ounass.ae/</t>
+          <t>https://site-39.example/</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>OUNASS UAE | The Definitive Home of Luxury</t>
+          <t>موقع تجريبي 39</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2789,7 +2789,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://www.6thstreet.com/</t>
+          <t>https://site-40.example/</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.6thstreet.com/</t>
+          <t>https://site-40.example/</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -2819,7 +2819,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>ERROR: The request could not be satisfied</t>
+          <t>موقع تجريبي 40</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2846,7 +2846,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.goldenscent.com/</t>
+          <t>https://site-41.example/</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.goldenscent.com/</t>
+          <t>https://site-41.example/</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.nahdionline.com/</t>
+          <t>https://site-42.example/</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.nahdionline.com/</t>
+          <t>https://site-42.example/</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>ERROR: The request could not be satisfied</t>
+          <t>موقع تجريبي 42</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2963,7 +2963,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.virginmegastore.ae/</t>
+          <t>https://site-43.example/</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -2976,12 +2976,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.virginmegastore.ae/en</t>
+          <t>https://site-43.example/en</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.virginmegastore.ae/ → https://www.virginmegastore.ae/en</t>
+          <t>https://site-43.example/ → https://site-43.example/en</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Virgin Megastore | Shop Online for Tech, Toys, Home Decor &amp; More</t>
+          <t>موقع تجريبي 43</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -3026,7 +3026,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://www.luluhypermarket.com/</t>
+          <t>https://site-44.example/</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.luluhypermarket.com/</t>
+          <t>https://site-44.example/</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -3056,7 +3056,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Attention Required! | Cloudflare</t>
+          <t>موقع تجريبي 44</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -3083,7 +3083,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://www.carrefourksa.com/</t>
+          <t>https://site-45.example/</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
@@ -3108,7 +3108,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://www.basharacare.com/</t>
+          <t>https://site-46.example/</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -3121,12 +3121,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.basharacare.com/ae_en</t>
+          <t>https://site-46.example/ae_en</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://www.basharacare.com/ → https://www.basharacare.com/ae_en</t>
+          <t>https://site-46.example/ → https://site-46.example/ae_en</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -3172,7 +3172,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.whites.net/</t>
+          <t>https://site-47.example/</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3185,12 +3185,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.whites.sa/ar-sa</t>
+          <t>https://site-48.example/ar-sa</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://www.whites.net/ → https://www.whites.sa → https://www.whites.sa/ar-sa</t>
+          <t>https://site-47.example/ → https://site-48.example → https://site-48.example/ar-sa</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Whites | Makeup, Skincare &amp; Hair Care Products</t>
+          <t>موقع تجريبي 47</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -3235,7 +3235,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://salla.com/</t>
+          <t>https://site-49.example/</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://salla.com/</t>
+          <t>https://site-49.example/</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Just a moment...</t>
+          <t>موقع تجريبي 49</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -3292,7 +3292,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://zid.sa/</t>
+          <t>https://site-50.example/</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://zid.sa/</t>
+          <t>https://site-50.example/</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -3322,7 +3322,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Just a moment...</t>
+          <t>موقع تجريبي 50</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -3349,7 +3349,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://www.shopify.com/</t>
+          <t>https://site-51.example/</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.shopify.com/</t>
+          <t>https://site-51.example/</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -3379,7 +3379,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Shopify: The All-in-One Commerce Platform for Businesses - Shopify</t>
+          <t>موقع تجريبي 51</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -3408,7 +3408,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://www.amazon.sa/</t>
+          <t>https://site-52.example/</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.amazon.sa/</t>
+          <t>https://site-52.example/</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -3438,7 +3438,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>أمازون السعودية: تسوق أونلاين | أسعار مخفضة على الإلكترونيات، الأزياء، الجوالات، البقالة والمزيد</t>
+          <t>موقع تجريبي 52</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -3471,7 +3471,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://www.mumzworld.com/</t>
+          <t>https://site-53.example/</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.mumzworld.com/</t>
+          <t>https://site-53.example/</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>

</xml_diff>